<commit_message>
chore: import local project baseline
</commit_message>
<xml_diff>
--- a/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
+++ b/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\信息收集整理\医生画像仓库\99_资料来源\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EE12E6-AC9E-4E4B-9921-BE575405BC0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A85C5E-1A73-4254-B6E2-E62CCF338957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2803" uniqueCount="805">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2815" uniqueCount="819">
   <si>
     <t>序号</t>
   </si>
@@ -2494,7 +2494,61 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>https://www.gyfyyy.cn/cn/ylfw/czcx/</t>
+    <t>http://www.gzhtcm3.com/</t>
+  </si>
+  <si>
+    <t>http://www.gzhtcm3.com/wsjs/zzts.htm</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.gyfyyy.cn/cn/ks/</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.gy3y.cn/ks/team.html</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>广州医科大学附属第二医院</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.gyey.com/cn/index.html</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.gyey.com/cn/ks/team.html</t>
+  </si>
+  <si>
+    <t>广州医科大学附属脑科医院</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.gzbrain.cn/</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.gzbrain.cn/myzj/list.html</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.gzbrain.cn/myzj/list.aspx</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>广州医科大学附属脑科医院(江村院区)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>广州市中医院</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.gzszyy.com/patient/</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.gzszyy.com/expert/</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -4751,9 +4805,13 @@
       <c r="H28" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="I28" s="4"/>
+      <c r="I28" s="4" t="s">
+        <v>804</v>
+      </c>
       <c r="J28" s="2"/>
-      <c r="K28" s="4"/>
+      <c r="K28" s="6" t="s">
+        <v>805</v>
+      </c>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
@@ -4774,7 +4832,9 @@
       <c r="U28" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="V28" s="2"/>
+      <c r="V28" s="2" t="s">
+        <v>774</v>
+      </c>
       <c r="W28" s="2"/>
       <c r="X28" s="2" t="s">
         <v>36</v>
@@ -4797,7 +4857,7 @@
         <v>795</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>200</v>
+        <v>795</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>29</v>
@@ -5168,7 +5228,7 @@
         <v>232</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="L35" s="2" t="s">
         <v>56</v>
@@ -5200,7 +5260,9 @@
       <c r="U35" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="V35" s="2"/>
+      <c r="V35" s="2" t="s">
+        <v>774</v>
+      </c>
       <c r="W35" s="2"/>
       <c r="X35" s="2" t="s">
         <v>36</v>
@@ -5237,8 +5299,8 @@
       <c r="J36" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="K36" s="4" t="s">
-        <v>241</v>
+      <c r="K36" s="6" t="s">
+        <v>807</v>
       </c>
       <c r="L36" s="2" t="s">
         <v>99</v>
@@ -5270,7 +5332,9 @@
       <c r="U36" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="V36" s="2"/>
+      <c r="V36" s="2" t="s">
+        <v>774</v>
+      </c>
       <c r="W36" s="2"/>
       <c r="X36" s="2" t="s">
         <v>36</v>
@@ -5290,7 +5354,7 @@
         <v>38</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>246</v>
+        <v>808</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>247</v>
@@ -5301,9 +5365,13 @@
       <c r="H37" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="I37" s="4"/>
+      <c r="I37" s="6" t="s">
+        <v>809</v>
+      </c>
       <c r="J37" s="2"/>
-      <c r="K37" s="4"/>
+      <c r="K37" s="4" t="s">
+        <v>810</v>
+      </c>
       <c r="L37" s="2"/>
       <c r="M37" s="2"/>
       <c r="N37" s="2"/>
@@ -5324,7 +5392,9 @@
       <c r="U37" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="V37" s="2"/>
+      <c r="V37" s="2" t="s">
+        <v>774</v>
+      </c>
       <c r="W37" s="2"/>
       <c r="X37" s="2" t="s">
         <v>36</v>
@@ -5344,7 +5414,7 @@
         <v>152</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>250</v>
+        <v>811</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>250</v>
@@ -5355,9 +5425,13 @@
       <c r="H38" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="I38" s="4"/>
+      <c r="I38" s="6" t="s">
+        <v>812</v>
+      </c>
       <c r="J38" s="2"/>
-      <c r="K38" s="4"/>
+      <c r="K38" s="6" t="s">
+        <v>813</v>
+      </c>
       <c r="L38" s="2"/>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
@@ -5378,7 +5452,9 @@
       <c r="U38" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="V38" s="2"/>
+      <c r="V38" s="2" t="s">
+        <v>774</v>
+      </c>
       <c r="W38" s="2"/>
       <c r="X38" s="2" t="s">
         <v>36</v>
@@ -5398,7 +5474,7 @@
         <v>253</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>254</v>
+        <v>815</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>254</v>
@@ -5409,8 +5485,8 @@
       <c r="H39" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="I39" s="4" t="s">
-        <v>255</v>
+      <c r="I39" s="6" t="s">
+        <v>814</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>256</v>
@@ -5460,7 +5536,7 @@
         <v>152</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>259</v>
+        <v>816</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>259</v>
@@ -5471,14 +5547,14 @@
       <c r="H40" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="I40" s="4" t="s">
-        <v>260</v>
+      <c r="I40" s="6" t="s">
+        <v>817</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="K40" s="4" t="s">
-        <v>262</v>
+      <c r="K40" s="6" t="s">
+        <v>818</v>
       </c>
       <c r="L40" s="2" t="s">
         <v>121</v>
@@ -5508,7 +5584,9 @@
       <c r="U40" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="V40" s="2"/>
+      <c r="V40" s="2" t="s">
+        <v>774</v>
+      </c>
       <c r="W40" s="2"/>
       <c r="X40" s="2" t="s">
         <v>36</v>
@@ -10266,10 +10344,18 @@
     <hyperlink ref="K34" r:id="rId35" xr:uid="{CBA606A5-5B0F-43DF-B5C3-948742EEC118}"/>
     <hyperlink ref="I35" r:id="rId36" xr:uid="{C2310FEA-8ABA-4F25-8FF9-7D71210E3993}"/>
     <hyperlink ref="K35" r:id="rId37" xr:uid="{A9F3AB30-015F-4FAB-89B8-4EC9ACE9A77E}"/>
+    <hyperlink ref="K28" r:id="rId38" xr:uid="{54BD2142-FA34-477B-B70E-012D2533CCE1}"/>
+    <hyperlink ref="K36" r:id="rId39" xr:uid="{D4CA3E11-0AEF-405E-B890-D2EC6401988B}"/>
+    <hyperlink ref="I37" r:id="rId40" xr:uid="{BD44E353-0D73-44C3-BE51-49F863A80A43}"/>
+    <hyperlink ref="I38" r:id="rId41" xr:uid="{918311B4-1A9A-4B27-B1DF-49190DAD7DCB}"/>
+    <hyperlink ref="K38" r:id="rId42" xr:uid="{76CDEC4D-F3CC-4519-BE44-0FBF127BBF11}"/>
+    <hyperlink ref="I39" r:id="rId43" xr:uid="{FEEBBBC1-DAD3-4121-8B5D-9A86DD9BDF1F}"/>
+    <hyperlink ref="I40" r:id="rId44" xr:uid="{F77F7695-606D-41C9-909B-FC7D1F9D707B}"/>
+    <hyperlink ref="K40" r:id="rId45" xr:uid="{11323039-78C9-4934-853C-F9B51943B5D1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId38"/>
+    <tablePart r:id="rId46"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: record Issue #14 skip decision
</commit_message>
<xml_diff>
--- a/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
+++ b/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="R49d373928ea34840"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="R2e64559ab4d14d14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rd32e4cf610d043b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R99162c98ed094bdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="R97337de1f01c483d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="Rfbe00e9329484c48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="Rc866f7ea6e4443b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rdb3eb34c0d124b56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R2bb154708bb84831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="R9a6d50c6efba4d4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4046,12 +4046,14 @@
       <x:c r="U19" s="2" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="V19" s="2" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="W19" s="2"/>
-      <x:c r="X19" s="2" t="s">
-        <x:v>36</x:v>
+      <x:c r="V19" s="2" t="str">
+        <x:v>跳过-无全院官方目录入口</x:v>
+      </x:c>
+      <x:c r="W19" s="2" t="str">
+        <x:v>两URL=芳村急诊1人、集团1人（无芳村）；院区200+，18人非全院；未采集/未写总表；全院目录后复排。</x:v>
+      </x:c>
+      <x:c r="X19" s="2" t="str">
+        <x:v>2026-08-12</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
@@ -10066,55 +10068,55 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R316838eb524b49ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="R1ca4ed07b0f74aaf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="Rf9d0edd8f7c24643"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="R74965ece0f85480a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="Rd25944e367a94349"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="Rb1cd3b554d8044ab"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="R6c629b99a0814964"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="R835126c6650a4f38"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="R9b1a2c365d7947b5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="R1f6dd2ca729b4bdb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="Rbd341694943349fe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="R06bebf0dc42e4a4c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R28983e3a0cbc479c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="R202652a4d40f4ddb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="R38cf907f5a404aa8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="Rbfce05d6658f47f7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="R6c16c8a4a09d4c6a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="R4fd9f38bc2fc47d9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R2817a1095d0e407e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="R95e0166675354db6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="Rf858e119d50f4346"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="R6d24999fd2c64c7a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="R59208fd2fb16417c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Rbc29d9aba4d04252"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="R949fc803423f4fbc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R59a0a70412274464"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="R3da6309250884d71"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R7e5fd2f8a8924cad"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R0318dc724767441b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R6a73bd3739194eef"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="Rf200c3671b264636"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R63a2b4e815d04944"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R275e6cc2f2ed4552"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="R4c1457d09d0e4dfd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rf4752c87ae9f46ff"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="Rb57dee9bbdfc4f49"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R02c1fe92b7ec44a6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="R26452fa3e66b4d81"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="R27320e242863491c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="Ra47b14f6946e45e9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="Rb9b70c9437b64c86"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="R601daeb91cda4d34"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="R2865e1ec7a2c4e74"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R6d6d2b2a57784afc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="R733b894ddb4b4b06"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R677b9792ecbb4628"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="Rca596f49f2114c3e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R9a959bfdd5184d3f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="Rcf0bd81adf8441ba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="R7c324eb12c6b4500"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="R9af0fc2d712b4696"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="Rcd68994248d44602"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="Rdada0108f1b14bf1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="R301791c03cb14cc3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="R429fcafab0694590"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="Rf5938269171546a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="Rd4ae9d3adf0440bd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R4fd060fdb3d04133"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="R5e129882c77f4993"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="Rc6d3de267c7b4a95"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R561f8e2967bf4ce9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="R5a7c8d77a55a4528"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Rec43899055514aba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R158d8b523f204911"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="R5e145ac87b584fda"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="R62690551a5be43ae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="R4cded82bb0094c39"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Rdc606b4c78ce4849"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Re0fdf24ad8f14c52"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Ra7dc41f509ce49a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R1cf2ded07d5e46e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="Rd6da9995e13941cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="Red2de00e44f64abd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R7d5c7350f33d4f18"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R149ba87370f34f9c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="R5cb89d6b10f544cd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R40ce36ba29154228"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R60b9b99504fe461b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="Ra41ee7ac1ad04d33"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="R894ee2dda8954561"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R4882b0870369433a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R2bf8727aa1a444fb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="Ra2da2a19b4ed4050"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="Rb02df562848249b8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R05254e76458a48b2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="Rda1dff60cde64812"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="R88fab0e2ccb54d98"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Rcd68c2e5163340ab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="Racf881a6519340ea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="Rcd04d9be988b45e3"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R761825f8873f4969"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b1d460238f493c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10393,7 +10395,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59bf6e7277304d93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9767b471b5b4057"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13060,7 +13062,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e73fdc73a0d4fc2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a94d0391e624cf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13116,7 +13118,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb30715261c54b6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re07780da93134424"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13188,7 +13190,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02ca08b7d42e4a16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb95683dfe12e4190"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record Issue #14 campus scope gate (#16)
* docs: record Issue 14 campus scope gate

* docs: record Issue #14 skip decision

---------

Co-authored-by: xtzhou247 <276638174+xtzhou247@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
+++ b/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="R49d373928ea34840"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="R2e64559ab4d14d14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rd32e4cf610d043b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R99162c98ed094bdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="R97337de1f01c483d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="Rfbe00e9329484c48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="Rc866f7ea6e4443b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rdb3eb34c0d124b56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R2bb154708bb84831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="R9a6d50c6efba4d4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4046,12 +4046,14 @@
       <x:c r="U19" s="2" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="V19" s="2" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="W19" s="2"/>
-      <x:c r="X19" s="2" t="s">
-        <x:v>36</x:v>
+      <x:c r="V19" s="2" t="str">
+        <x:v>跳过-无全院官方目录入口</x:v>
+      </x:c>
+      <x:c r="W19" s="2" t="str">
+        <x:v>两URL=芳村急诊1人、集团1人（无芳村）；院区200+，18人非全院；未采集/未写总表；全院目录后复排。</x:v>
+      </x:c>
+      <x:c r="X19" s="2" t="str">
+        <x:v>2026-08-12</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
@@ -10066,55 +10068,55 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R316838eb524b49ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="R1ca4ed07b0f74aaf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="Rf9d0edd8f7c24643"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="R74965ece0f85480a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="Rd25944e367a94349"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="Rb1cd3b554d8044ab"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="R6c629b99a0814964"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="R835126c6650a4f38"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="R9b1a2c365d7947b5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="R1f6dd2ca729b4bdb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="Rbd341694943349fe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="R06bebf0dc42e4a4c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R28983e3a0cbc479c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="R202652a4d40f4ddb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="R38cf907f5a404aa8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="Rbfce05d6658f47f7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="R6c16c8a4a09d4c6a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="R4fd9f38bc2fc47d9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R2817a1095d0e407e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="R95e0166675354db6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="Rf858e119d50f4346"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="R6d24999fd2c64c7a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="R59208fd2fb16417c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Rbc29d9aba4d04252"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="R949fc803423f4fbc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R59a0a70412274464"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="R3da6309250884d71"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R7e5fd2f8a8924cad"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R0318dc724767441b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R6a73bd3739194eef"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="Rf200c3671b264636"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R63a2b4e815d04944"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R275e6cc2f2ed4552"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="R4c1457d09d0e4dfd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rf4752c87ae9f46ff"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="Rb57dee9bbdfc4f49"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R02c1fe92b7ec44a6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="R26452fa3e66b4d81"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="R27320e242863491c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="Ra47b14f6946e45e9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="Rb9b70c9437b64c86"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="R601daeb91cda4d34"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="R2865e1ec7a2c4e74"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R6d6d2b2a57784afc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="R733b894ddb4b4b06"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R677b9792ecbb4628"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="Rca596f49f2114c3e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R9a959bfdd5184d3f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="Rcf0bd81adf8441ba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="R7c324eb12c6b4500"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="R9af0fc2d712b4696"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="Rcd68994248d44602"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="Rdada0108f1b14bf1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="R301791c03cb14cc3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="R429fcafab0694590"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="Rf5938269171546a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="Rd4ae9d3adf0440bd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R4fd060fdb3d04133"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="R5e129882c77f4993"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="Rc6d3de267c7b4a95"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R561f8e2967bf4ce9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="R5a7c8d77a55a4528"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Rec43899055514aba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R158d8b523f204911"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="R5e145ac87b584fda"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="R62690551a5be43ae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="R4cded82bb0094c39"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Rdc606b4c78ce4849"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Re0fdf24ad8f14c52"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Ra7dc41f509ce49a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R1cf2ded07d5e46e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="Rd6da9995e13941cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="Red2de00e44f64abd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R7d5c7350f33d4f18"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R149ba87370f34f9c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="R5cb89d6b10f544cd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R40ce36ba29154228"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R60b9b99504fe461b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="Ra41ee7ac1ad04d33"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="R894ee2dda8954561"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R4882b0870369433a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R2bf8727aa1a444fb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="Ra2da2a19b4ed4050"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="Rb02df562848249b8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R05254e76458a48b2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="Rda1dff60cde64812"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="R88fab0e2ccb54d98"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Rcd68c2e5163340ab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="Racf881a6519340ea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="Rcd04d9be988b45e3"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R761825f8873f4969"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b1d460238f493c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10393,7 +10395,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59bf6e7277304d93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9767b471b5b4057"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13060,7 +13062,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e73fdc73a0d4fc2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a94d0391e624cf4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13116,7 +13118,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb30715261c54b6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re07780da93134424"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13188,7 +13190,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02ca08b7d42e4a16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb95683dfe12e4190"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(issue-29): record GYEY access block
</commit_message>
<xml_diff>
--- a/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
+++ b/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="Rfbe00e9329484c48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="Rc866f7ea6e4443b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rdb3eb34c0d124b56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R2bb154708bb84831"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="R9a6d50c6efba4d4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="R9d6c026564994f5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="R965122bc7d9243da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rc0fee14ec9894c1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R46022a833cac4d21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="Rc7f4f802f54e4f24"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5102,7 +5102,7 @@
         <x:v>36</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="42" customHeight="1">
+    <x:row r="37" ht="60" customHeight="1">
       <x:c r="A37" s="2" t="s">
         <x:v>263</x:v>
       </x:c>
@@ -5150,16 +5150,20 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="S37" s="2"/>
-      <x:c r="T37" s="2"/>
-      <x:c r="U37" s="2" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="V37" s="2" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="W37" s="2"/>
-      <x:c r="X37" s="2" t="s">
-        <x:v>36</x:v>
+      <x:c r="T37" s="2" t="str">
+        <x:v>官网首页与 Issue #29 指定医生目录常规 GET 均返回 HTTP 403；响应页面标题为“您的访问请求可能对网站造成安全威胁，请求已被阻断。”未取得真实页面。禁止绕过站点安全拦截。</x:v>
+      </x:c>
+      <x:c r="U37" s="2" t="str">
+        <x:v>跳过本院；不绕过访问拦截；等待 owner 审计 Issue #29</x:v>
+      </x:c>
+      <x:c r="V37" s="2" t="str">
+        <x:v>跳过-访问拦截</x:v>
+      </x:c>
+      <x:c r="W37" s="2" t="str">
+        <x:v>2026-08-13 Codex 按 Issue #29 预先裁决执行：仅普通公开 HTTP GET，无挑战应答、验证码处理、浏览器指纹模拟、代理或第三方来源。未运行采集器，未写入总底表。证据见 Issue #29、WAF 报告与 ADR。</x:v>
+      </x:c>
+      <x:c r="X37" s="2" t="str">
+        <x:v>2026-08-13</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
@@ -10068,55 +10072,55 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R677b9792ecbb4628"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="Rca596f49f2114c3e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R9a959bfdd5184d3f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="Rcf0bd81adf8441ba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="R7c324eb12c6b4500"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="R9af0fc2d712b4696"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="Rcd68994248d44602"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="Rdada0108f1b14bf1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="R301791c03cb14cc3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="R429fcafab0694590"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="Rf5938269171546a1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="Rd4ae9d3adf0440bd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R4fd060fdb3d04133"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="R5e129882c77f4993"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="Rc6d3de267c7b4a95"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R561f8e2967bf4ce9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="R5a7c8d77a55a4528"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Rec43899055514aba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R158d8b523f204911"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="R5e145ac87b584fda"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="R62690551a5be43ae"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="R4cded82bb0094c39"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Rdc606b4c78ce4849"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Re0fdf24ad8f14c52"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Ra7dc41f509ce49a9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R1cf2ded07d5e46e6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="Rd6da9995e13941cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="Red2de00e44f64abd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R7d5c7350f33d4f18"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R149ba87370f34f9c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="R5cb89d6b10f544cd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R40ce36ba29154228"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R60b9b99504fe461b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="Ra41ee7ac1ad04d33"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="R894ee2dda8954561"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R4882b0870369433a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R2bf8727aa1a444fb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="Ra2da2a19b4ed4050"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="Rb02df562848249b8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R05254e76458a48b2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="Rda1dff60cde64812"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="R88fab0e2ccb54d98"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Rcd68c2e5163340ab"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="Racf881a6519340ea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="Rcd04d9be988b45e3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R4044a9c4e1ca468f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="Rb49900af14fd4721"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="Re8e0ff779ec24c16"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="R353f4bccb6024cc3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="R9846b63c6eda411d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="R33d26b88042a4679"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="Rb6324b838d914b02"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="Rbf0347b6adf4414e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="Rdc9d0621a17e4518"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="Rf1e32b74b8444a1f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="R38a889087d434af6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="R769dc5414bf3499b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R9c96705701624c24"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="Rf7e1fb82725c444d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="R60b6322216834f36"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R866ff2830b5d4609"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="R6bab108250a94705"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Rb6309be3c9944186"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R2753fe086e09493c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="Rff88087034ea4d12"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="R44f3cf1d3753484d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Rd5389feb365842c9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Rbf1da644c1ae4699"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="R630dfff9ca1b4ee9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Rdc0cf2ea6fb94b06"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R51640ccf1acb4c3b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="R59da4011c31e43b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R81668c0658804770"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R6224f69f4f314b3d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R1a06ed87f19140a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="R4eb9d5aab98d4a9d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R9ac7a414a102412c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="Re9c33e1537a54328"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="R6542ad29523c4e32"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rf3c93764109b45a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R4a92ff74d39b4177"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="Rf3cb103f7b004ff3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="Ra5170a45ba7c40e8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="R0723497e14a04efb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R53f197e4aec847a0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="R4c447dfd30894689"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="Rabe730b8c8b94942"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Ra459bebbe6584d03"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R1e2afbb3e6224125"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="Rcdc12b352a924608"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b1d460238f493c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7f17bc62c56470c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10395,7 +10399,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9767b471b5b4057"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ac9af835ff24b83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11239,7 +11243,7 @@
       <x:c r="H36" s="2"/>
       <x:c r="I36" s="2"/>
     </x:row>
-    <x:row r="37" ht="16.5">
+    <x:row r="37" ht="60" customHeight="1">
       <x:c r="A37" s="2" t="s">
         <x:v>25</x:v>
       </x:c>
@@ -11254,11 +11258,15 @@
       <x:c r="F37" s="2" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="G37" s="2" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="H37" s="2"/>
-      <x:c r="I37" s="2"/>
+      <x:c r="G37" s="2" t="str">
+        <x:v>跳过本院；不绕过访问拦截；等待 owner 审计 Issue #29</x:v>
+      </x:c>
+      <x:c r="H37" s="2" t="str">
+        <x:v>跳过-访问拦截</x:v>
+      </x:c>
+      <x:c r="I37" s="2" t="str">
+        <x:v>官网首页与医生目录均 HTTP 403，页面提示访问请求可能造成安全威胁并已阻断；仅普通 GET，未取得真实页面，未运行采集器，未写入总底表。</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="16.5">
       <x:c r="A38" s="2" t="s">
@@ -13062,7 +13070,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a94d0391e624cf4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0474317d56504f54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13118,7 +13126,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re07780da93134424"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc374a3a6b4554bc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13190,7 +13198,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb95683dfe12e4190"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8beac2faabb44a81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(issue-29): record GYEY access block (#30)
Co-authored-by: xtzhou247 <276638174+xtzhou247@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
+++ b/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="Rfbe00e9329484c48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="Rc866f7ea6e4443b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rdb3eb34c0d124b56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R2bb154708bb84831"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="R9a6d50c6efba4d4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="R9d6c026564994f5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="R965122bc7d9243da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rc0fee14ec9894c1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R46022a833cac4d21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="Rc7f4f802f54e4f24"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5102,7 +5102,7 @@
         <x:v>36</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="42" customHeight="1">
+    <x:row r="37" ht="60" customHeight="1">
       <x:c r="A37" s="2" t="s">
         <x:v>263</x:v>
       </x:c>
@@ -5150,16 +5150,20 @@
         <x:v>268</x:v>
       </x:c>
       <x:c r="S37" s="2"/>
-      <x:c r="T37" s="2"/>
-      <x:c r="U37" s="2" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="V37" s="2" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="W37" s="2"/>
-      <x:c r="X37" s="2" t="s">
-        <x:v>36</x:v>
+      <x:c r="T37" s="2" t="str">
+        <x:v>官网首页与 Issue #29 指定医生目录常规 GET 均返回 HTTP 403；响应页面标题为“您的访问请求可能对网站造成安全威胁，请求已被阻断。”未取得真实页面。禁止绕过站点安全拦截。</x:v>
+      </x:c>
+      <x:c r="U37" s="2" t="str">
+        <x:v>跳过本院；不绕过访问拦截；等待 owner 审计 Issue #29</x:v>
+      </x:c>
+      <x:c r="V37" s="2" t="str">
+        <x:v>跳过-访问拦截</x:v>
+      </x:c>
+      <x:c r="W37" s="2" t="str">
+        <x:v>2026-08-13 Codex 按 Issue #29 预先裁决执行：仅普通公开 HTTP GET，无挑战应答、验证码处理、浏览器指纹模拟、代理或第三方来源。未运行采集器，未写入总底表。证据见 Issue #29、WAF 报告与 ADR。</x:v>
+      </x:c>
+      <x:c r="X37" s="2" t="str">
+        <x:v>2026-08-13</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
@@ -10068,55 +10072,55 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R677b9792ecbb4628"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="Rca596f49f2114c3e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R9a959bfdd5184d3f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="Rcf0bd81adf8441ba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="R7c324eb12c6b4500"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="R9af0fc2d712b4696"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="Rcd68994248d44602"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="Rdada0108f1b14bf1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="R301791c03cb14cc3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="R429fcafab0694590"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="Rf5938269171546a1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="Rd4ae9d3adf0440bd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R4fd060fdb3d04133"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="R5e129882c77f4993"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="Rc6d3de267c7b4a95"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R561f8e2967bf4ce9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="R5a7c8d77a55a4528"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Rec43899055514aba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R158d8b523f204911"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="R5e145ac87b584fda"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="R62690551a5be43ae"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="R4cded82bb0094c39"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Rdc606b4c78ce4849"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Re0fdf24ad8f14c52"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Ra7dc41f509ce49a9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R1cf2ded07d5e46e6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="Rd6da9995e13941cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="Red2de00e44f64abd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R7d5c7350f33d4f18"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R149ba87370f34f9c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="R5cb89d6b10f544cd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R40ce36ba29154228"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R60b9b99504fe461b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="Ra41ee7ac1ad04d33"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="R894ee2dda8954561"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R4882b0870369433a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R2bf8727aa1a444fb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="Ra2da2a19b4ed4050"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="Rb02df562848249b8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R05254e76458a48b2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="Rda1dff60cde64812"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="R88fab0e2ccb54d98"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Rcd68c2e5163340ab"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="Racf881a6519340ea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="Rcd04d9be988b45e3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R4044a9c4e1ca468f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="Rb49900af14fd4721"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="Re8e0ff779ec24c16"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="R353f4bccb6024cc3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="R9846b63c6eda411d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="R33d26b88042a4679"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="Rb6324b838d914b02"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="Rbf0347b6adf4414e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="Rdc9d0621a17e4518"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="Rf1e32b74b8444a1f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="R38a889087d434af6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="R769dc5414bf3499b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R9c96705701624c24"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="Rf7e1fb82725c444d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="R60b6322216834f36"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R866ff2830b5d4609"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="R6bab108250a94705"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Rb6309be3c9944186"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R2753fe086e09493c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="Rff88087034ea4d12"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="R44f3cf1d3753484d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Rd5389feb365842c9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Rbf1da644c1ae4699"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="R630dfff9ca1b4ee9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Rdc0cf2ea6fb94b06"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R51640ccf1acb4c3b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="R59da4011c31e43b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R81668c0658804770"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R6224f69f4f314b3d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R1a06ed87f19140a1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="R4eb9d5aab98d4a9d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R9ac7a414a102412c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="Re9c33e1537a54328"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="R6542ad29523c4e32"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rf3c93764109b45a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R4a92ff74d39b4177"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="Rf3cb103f7b004ff3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="Ra5170a45ba7c40e8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="R0723497e14a04efb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R53f197e4aec847a0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="R4c447dfd30894689"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="Rabe730b8c8b94942"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Ra459bebbe6584d03"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R1e2afbb3e6224125"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="Rcdc12b352a924608"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5b1d460238f493c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7f17bc62c56470c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10395,7 +10399,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9767b471b5b4057"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ac9af835ff24b83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11239,7 +11243,7 @@
       <x:c r="H36" s="2"/>
       <x:c r="I36" s="2"/>
     </x:row>
-    <x:row r="37" ht="16.5">
+    <x:row r="37" ht="60" customHeight="1">
       <x:c r="A37" s="2" t="s">
         <x:v>25</x:v>
       </x:c>
@@ -11254,11 +11258,15 @@
       <x:c r="F37" s="2" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="G37" s="2" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="H37" s="2"/>
-      <x:c r="I37" s="2"/>
+      <x:c r="G37" s="2" t="str">
+        <x:v>跳过本院；不绕过访问拦截；等待 owner 审计 Issue #29</x:v>
+      </x:c>
+      <x:c r="H37" s="2" t="str">
+        <x:v>跳过-访问拦截</x:v>
+      </x:c>
+      <x:c r="I37" s="2" t="str">
+        <x:v>官网首页与医生目录均 HTTP 403，页面提示访问请求可能造成安全威胁并已阻断；仅普通 GET，未取得真实页面，未运行采集器，未写入总底表。</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="16.5">
       <x:c r="A38" s="2" t="s">
@@ -13062,7 +13070,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a94d0391e624cf4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0474317d56504f54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13118,7 +13126,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re07780da93134424"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc374a3a6b4554bc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13190,7 +13198,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb95683dfe12e4190"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8beac2faabb44a81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(issue-39): verify and skip duplicate Huangpu directory
</commit_message>
<xml_diff>
--- a/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
+++ b/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="R9d6c026564994f5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="R965122bc7d9243da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rc0fee14ec9894c1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R46022a833cac4d21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="Rc7f4f802f54e4f24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="Rf35e6269431e4304"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="Rcc579bebcdd446b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rbd5eb8b909bc47a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R737b89720af04288"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="R40e26bf4548c4930"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3376,8 +3376,8 @@
       <x:c r="U9" s="2" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="V9" s="2" t="s">
-        <x:v>66</x:v>
+      <x:c r="V9" s="2" t="str">
+        <x:v>跳过-与序号7同源目录已全量入库</x:v>
       </x:c>
       <x:c r="W9" s="2"/>
       <x:c r="X9" s="2" t="s">
@@ -10072,55 +10072,55 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R4044a9c4e1ca468f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="Rb49900af14fd4721"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="Re8e0ff779ec24c16"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="R353f4bccb6024cc3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="R9846b63c6eda411d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="R33d26b88042a4679"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="Rb6324b838d914b02"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="Rbf0347b6adf4414e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="Rdc9d0621a17e4518"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="Rf1e32b74b8444a1f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="R38a889087d434af6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="R769dc5414bf3499b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R9c96705701624c24"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="Rf7e1fb82725c444d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="R60b6322216834f36"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R866ff2830b5d4609"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="R6bab108250a94705"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Rb6309be3c9944186"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R2753fe086e09493c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="Rff88087034ea4d12"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="R44f3cf1d3753484d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Rd5389feb365842c9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Rbf1da644c1ae4699"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="R630dfff9ca1b4ee9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Rdc0cf2ea6fb94b06"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R51640ccf1acb4c3b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="R59da4011c31e43b5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R81668c0658804770"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R6224f69f4f314b3d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R1a06ed87f19140a1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="R4eb9d5aab98d4a9d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R9ac7a414a102412c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="Re9c33e1537a54328"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="R6542ad29523c4e32"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rf3c93764109b45a4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R4a92ff74d39b4177"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="Rf3cb103f7b004ff3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="Ra5170a45ba7c40e8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="R0723497e14a04efb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R53f197e4aec847a0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="R4c447dfd30894689"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="Rabe730b8c8b94942"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Ra459bebbe6584d03"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R1e2afbb3e6224125"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="Rcdc12b352a924608"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R5c5cb511f9174bb5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="R816b2b1b49af4372"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R2fbc8c34401d4696"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="R70515154b72c484d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="Rd6961ada84a24cab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="Ra8bfc8fad18d4af2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="R7029fdb0c7034d46"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="R2d84657936884abe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="Rbdbdf2f19b1a4919"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="R54177e6efed64abe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="R75b3b73fd9d242b4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="R4d94383b46524367"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R3bc2b2c67d1341c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="R121519b2079144bc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="R2bb716764146401f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R725e7f3d53ed4142"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="Rffe98eb621774859"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="R533fe849af00449a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="R2f58a6e5452444c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="R9f69ee3ac01f43b9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="Rb028a6fbd72d4d28"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Rcc8098f036ec40d3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Rfd0e05f16e10407d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Rb5f1cff263eb4ef7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="R4b18753b1a2c4e90"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="Rd9e45dbc3e7749df"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="Re0f8e023cd2e4417"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="Rb6a438b94f724e6c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R5a20f01e46b640f5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R0a0ec7c60d6c4436"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="Ra192084f6e484ba9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R0ee6307f9a3d44f5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R43209ec63c0b4154"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="R4db21bde1e3a400b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rfd9dc3c6512b43ec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R7910902f71ae4563"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R4a12cff2ac7c4cc7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="R5a2d0f96c539415f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="Rc1cb169b2ed7465f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="Rb5fb01bbe7474d41"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="R2619a68161764b3b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="Re09fd8bd35db4710"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Rb055ebba446948fc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="Rfd4901d499ba46e5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="R5ee1bd6c8a2c4ee9"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7f17bc62c56470c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R755524f7b0964f8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10399,7 +10399,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ac9af835ff24b83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e420795aea544db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13070,7 +13070,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0474317d56504f54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R606f5c685f4744a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13126,7 +13126,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc374a3a6b4554bc0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1911f1256b474a75"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13198,7 +13198,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8beac2faabb44a81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R730f1bbf038a4738"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete GYFYYY doctor photo backfill
</commit_message>
<xml_diff>
--- a/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
+++ b/医生画像仓库/99_资料来源/珠三角三甲医院官网入口台账.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="R2ab4198e6161431f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="R7f0d2d9028f94b78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="Rdccb00b49d3a4bce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R4f2881f123a44714"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="R334e36c6f8f54623"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入口台账" sheetId="1" r:id="R35a96fc4e68849fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市汇总" sheetId="2" r:id="Re4ac96476d09442e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工复核清单" sheetId="3" r:id="R725db6e170d049a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="Rf91c64cea8d74035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" r:id="Raeef376cf40c490d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3869,11 +3869,11 @@
       <x:c r="S16" s="2" t="s">
         <x:v>142</x:v>
       </x:c>
-      <x:c r="T16" s="2" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="U16" s="2" t="s">
-        <x:v>65</x:v>
+      <x:c r="T16" s="2" t="str">
+        <x:v>入口锚文本：专家介绍；管理员裁决跳过（军队医院，2026-08-17）</x:v>
+      </x:c>
+      <x:c r="U16" s="2" t="str">
+        <x:v>跳过</x:v>
       </x:c>
       <x:c r="V16" s="2" t="s">
         <x:v>66</x:v>
@@ -10089,55 +10089,55 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R33ffe6539f694917"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="R36c21bb35cea42c3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="Rc66d91c0c35d4d9a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="R030f50c53ea541b1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="R21d4bf280c194bb6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="R40a7c891a40b45d1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="R1dec603ce7bc4442"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="R58eab9b80d2e48aa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="Re1b3f238751249e7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="Ra970982095f946f7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="Rf3517abf58164de7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="Rd24b1909ccb74f07"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R601ec40c61494945"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="R22b1120e94af448b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="R711f65b57d3c481c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R664067dfb2fc4734"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="Rc6a5c2a1787d4d0d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Ra997f5e3528a4f61"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="Rea5e0ab37ef94eca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="Ra92777122ace4fa8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="Rdaf850a540994fa3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Rc85eed91b6144c20"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Ra23d89b8997946dc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Rc1060bd494074cbf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Rf7ab0c0783b94e6a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R48107b64042b4726"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="Rc37d29bef5314698"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="Rf69c924e779d4d52"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R2540eba63ed74ea6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R34b7bc34ef9845ea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="Rca14e5f1547c4f03"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R5933b7a1c7754cb0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R9dfc103acc5b42b2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="Ree6b52da1e0e4ead"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="R5ab94717331449b9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R6dea6cb3368049eb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R0e453b2d8a6446d2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="R125cbeaceead4c41"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="Rea06ff48f8474e22"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="Rd185949d182e491b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="Rbad2cdb4f39f4942"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="R4fc587f1b8c44278"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="R23dc279fa1dd46d8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R8f2a81d061df49ae"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="R36ff7854aadb465e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="R613fe9d9b6cb4cda"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="Rbd7e3f60bf554d1a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R4fed7d6460dd40f7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="R136946bb5764437d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="R78d3d3f8b62d4b86"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="R4be128aee86144a3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="Ra305d03147914d05"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="R6281ab4f3f5e49f5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="R726407611f4348d9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="Rc9cc13c2db4a4792"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="Ra3e6bd4daa4240ad"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="R4b4842ab5fba413d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="R4a64e278c3d74284"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="Rcffe16ceb53e4a54"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="Ra465be85ba5d455b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R83633dd487a84111"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="Rd3fa6611a7ca407a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="R338456d823954414"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="Ra82d65eaf79e4d1a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="R90d0c80c81194da1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="R668c5ff40575428f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Re0c5d096b2f14a1f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="Rfb9e2443a6a04694"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Rbfdbe7c2ffaf4566"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="Rc6316dbd6c0142f4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R157868301bc346de"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="R2232a73acf1e4d4f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R11b26225e2e8460d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="R93309c90caf74e09"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R646c8032f9014c55"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="R8a67db325f5f445f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="Rad71da3aa6794bfb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="R87b95a42b1c14b98"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="R01536b0440d14f93"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rdeaeb229aa7d4ee8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="R66cd7749dcc54689"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="Red24c9777efe4dee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="R60ec3ac2c8f24fd1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="Rfd584c02cd2446cb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R613b93de76f84ebf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="R4dbc6c23c59e47e0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="R8111685614984d76"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Rfbc3be5f60c84a5f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="Rac1a26b07dac4ef9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="R16fdfd2a36b547f3"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R149744666abf47a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d8e5008a1fc410e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10416,7 +10416,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra227091762b6444d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d48e9a0bb444015"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13087,7 +13087,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05ba0b38dd1c4ef4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb26dfecb62214332"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13143,7 +13143,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fddebc214844613"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re58d9c4f0b2842b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13215,7 +13215,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28f0d5dbe81543f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R435137deb8204811"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>